<commit_message>
Update mosip_master XLSX files
Updated multiple binary master spreadsheets under mosip_master/xlsx (applicant_valid_document, blocklisted_words, daysofweek_list, doc_category, doc_type, dynamic_field, identity_schema, language, loc_hierarchy_list, loc_holiday, location, reason_category, reason_list, reg_center_type, reg_working_nonworking, registration_center, registration_center_h, template, template_type, title, ui_spec, valid_document, zone, zone_user, zone_user_h). These are content/data updates to the repository's reference XLSX files.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/identity_schema.xlsx
+++ b/mosip_master/xlsx/identity_schema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\Mosip\mosip-data\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Workspace\SLUDI\MVP\Training\MaterData\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E632B33-EFBA-45CC-B1A2-807AF397E164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45700110-692E-41FA-B8A2-59EF37158CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,10 +79,10 @@
   </si>
   <si>
     <t>{
-	"$schema": "http:\/\/json-schema.org\/draft-07\/schema#",
-	"description": "MOSIP Sample identity",
+	"$schema": "http://json-schema.org/draft-07/schema#",
+	"description": "SLUDI identity schema for MOSIP ID Repository",
 	"additionalProperties": false,
-	"title": "MOSIP identity",
+	"title": "SLUDI identity",
 	"type": "object",
 	"definitions": {
 		"simpleType": {
@@ -109,6 +109,11 @@
 		"documentType": {
 			"additionalProperties": false,
 			"type": "object",
+			"required": [
+				"format",
+				"type",
+				"value"
+			],
 			"properties": {
 				"format": {
 					"type": "string"
@@ -130,6 +135,11 @@
 		"biometricsType": {
 			"additionalProperties": false,
 			"type": "object",
+			"required": [
+				"format",
+				"version",
+				"value"
+			],
 			"properties": {
 				"format": {
 					"type": "string"
@@ -150,88 +160,471 @@
 			"type": "object",
 			"required": [
 				"IDSchemaVersion",
-				"fullName",
+				"name",
+				"surname",
 				"dateOfBirth",
 				"gender",
+				"placeOfBirth",
+				"divisionalSecretariatOfBirth",
 				"addressLine1",
-				"addressLine2",
-				"addressLine3",
-				"region",
 				"province",
-				"city",
-				"zone",
+				"district",
+				"divisionalSecretariat",
+				"grammaNiladhari",
 				"postalCode",
-				"phone",
-				"email",
-				"proofOfIdentity",
+				"applicantSignature",
 				"individualBiometrics"
 			],
 			"properties": {
-				"proofOfAddress": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"gender": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"city": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"postalCode": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^[(?i)A-Z0-9]{5}$|^NA$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
+				"IDSchemaVersion": {
+					"bioAttributes": [],
+					"fieldCategory": "none",
+					"format": "none",
+					"type": "number",
+					"fieldType": "default",
+					"minimum": 0
+				},
+				"UIN": {
+					"bioAttributes": [],
+					"fieldCategory": "none",
 					"format": "none",
 					"type": "string",
 					"fieldType": "default"
 				},
-				"proofOfException-1": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
+				"familyName": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{3,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"name": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{3,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"surname": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{3,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"gender": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"dateOfBirth": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"placeOfBirth": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{2,128}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"divisionalSecretariatOfBirth": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"deathDeclared": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(yes|no)$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"dateOfDeath": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"addressLine1": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,128}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"addressLine2": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"addressLine3": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"province": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"district": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"divisionalSecretariat": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"grammaNiladhari": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"postalCode": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^[0-9]{5}$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"currentAddressLine1": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentAddressLine2": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentAddressLine3": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentProvince": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentDistrict": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentDivisionalSecretariat": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentGramaNiladhari": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentPostalCode": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^$|^[0-9]{5}$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
 				},
 				"referenceIdentityNumber": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^([0-9]{10,30})$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?:\\d{9}[VXvx]|\\d{12})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "kyc",
 					"format": "kyc",
 					"type": "string",
 					"fieldType": "default"
+				},
+				"phone": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(0?7[0-9]{8})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"email": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"preferredLang": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "dynamic"
+				},
+				"applicantSignature": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"subType": "POI",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfDateOfBirth": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfAddress": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfIdentity": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfRelationship": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfException": {
+					"bioAttributes": [],
+					"fieldCategory": "evidence",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
 				},
 				"individualBiometrics": {
 					"bioAttributes": [
@@ -252,109 +645,49 @@
 					"fieldCategory": "pvt",
 					"format": "none",
 					"fieldType": "default",
-					"$ref": "#\/definitions\/biometricsType"
-				},
-				"province": {
+					"$ref": "#/definitions/biometricsType"
+				},
+				"individualAuthBiometrics": {
 					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"zone": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"proofOfDateOfBirth": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"addressLine1": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"addressLine2": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"residenceStatus": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "kyc",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"addressLine3": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"email": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
+						"leftEye",
+						"rightEye",
+						"rightIndex",
+						"rightLittle",
+						"rightRing",
+						"rightMiddle",
+						"leftIndex",
+						"leftLittle",
+						"leftRing",
+						"leftMiddle",
+						"leftThumb",
+						"rightThumb",
+						"face"
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/biometricsType"
+				},
+				"introducerRID": {
+					"bioAttributes": [],
+					"fieldCategory": "evidence",
 					"format": "none",
 					"type": "string",
 					"fieldType": "default"
 				},
-				"introducerRID": {
-					"bioAttributes": [
-					],
+				"introducerUIN": {
+					"bioAttributes": [],
 					"fieldCategory": "evidence",
 					"format": "none",
 					"type": "string",
 					"fieldType": "default"
+				},
+				"introducerName": {
+					"bioAttributes": [],
+					"fieldCategory": "evidence",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
 				},
 				"introducerBiometrics": {
 					"bioAttributes": [
@@ -375,206 +708,8 @@
 					"fieldCategory": "pvt",
 					"format": "none",
 					"fieldType": "default",
-					"$ref": "#\/definitions\/biometricsType"
-				},
-				"fullName": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"dateOfBirth": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])\/([0][1-9]|1[0-2])\/([0][1-9]|[1-2][0-9]|3[01])$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"individualAuthBiometrics": {
-					"bioAttributes": [
-						"leftEye",
-						"rightEye",
-						"rightIndex",
-						"rightLittle",
-						"rightRing",
-						"rightMiddle",
-						"leftIndex",
-						"leftLittle",
-						"leftRing",
-						"leftMiddle",
-						"leftThumb",
-						"rightThumb",
-						"face"
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/biometricsType"
-				},
-				"introducerUIN": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"proofOfIdentity": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"IDSchemaVersion": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "none",
-					"format": "none",
-					"type": "number",
-					"fieldType": "default",
-					"minimum": 0
-				},
-				"proofOfException": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"phone": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^[+]*([0-9]{1})([0-9]{9})$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"introducerName": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"proofOfRelationship": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"UIN": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "none",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"preferredLang": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"type": "string",
-					"fieldType": "dynamic"
-				},
-				"region": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"introducerInfoToken": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "evidence",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "deceasedInformer": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "evidence",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "deceasedDeclarationDate": {
-                    "bioAttributes": [
-                    ],
-                    "validators": [
-                        {
-                            "validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
-                            "arguments": [
-                            ],
-                            "type": "regex"
-                        }
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "declaredAsDeceased": {
-                    "bioAttributes": [
-                    ],
-                    "validators": [
-                        {
-                            "validator": "^(Y|N)$",
-                            "arguments": [
-                            ],
-                            "type": "regex"
-                        }
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "typeOfDeath": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                }
+					"$ref": "#/definitions/biometricsType"
+				}
 			}
 		}
 	}
@@ -670,9 +805,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -710,7 +845,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -816,7 +951,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -958,7 +1093,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -967,23 +1102,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AMJ3"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.453125" style="1"/>
-    <col min="2" max="2" width="8.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="11.54296875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.453125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.44140625" style="1"/>
+    <col min="2" max="2" width="8.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="31" style="1" customWidth="1"/>
-    <col min="6" max="6" width="53.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7265625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="53.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.44140625" style="2" customWidth="1"/>
     <col min="9" max="9" width="10" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" style="2"/>
-    <col min="11" max="1023" width="8.453125" style="1"/>
-    <col min="1024" max="1024" width="11.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.44140625" style="2"/>
+    <col min="11" max="1023" width="8.44140625" style="1"/>
+    <col min="1024" max="1024" width="11.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1015,7 +1150,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1047,7 +1182,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="F3" s="5"/>
     </row>

</xml_diff>

<commit_message>
Update master XLSX files; add two new files
Updated multiple master spreadsheet files under mosip_master/xlsx (various .xlsx files modified). Added two new spreadsheet files: mosip_master/xlsx/doc_category_new.xlsx and mosip_master/xlsx/loc_holiday_new.xlsx. These are binary master-data spreadsheet updates to refresh categories, holidays, and related master lists.
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/identity_schema.xlsx
+++ b/mosip_master/xlsx/identity_schema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mosip-data-fix-license\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Workspace\SLUDI\MVP\Training\MaterData\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D433272-7AFA-4B99-A709-E889310C4AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45700110-692E-41FA-B8A2-59EF37158CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,10 +79,10 @@
   </si>
   <si>
     <t>{
-	"$schema": "http:\/\/json-schema.org\/draft-07\/schema#",
-	"description": "MOSIP Sample identity",
+	"$schema": "http://json-schema.org/draft-07/schema#",
+	"description": "SLUDI identity schema for MOSIP ID Repository",
 	"additionalProperties": false,
-	"title": "MOSIP identity",
+	"title": "SLUDI identity",
 	"type": "object",
 	"definitions": {
 		"simpleType": {
@@ -109,6 +109,11 @@
 		"documentType": {
 			"additionalProperties": false,
 			"type": "object",
+			"required": [
+				"format",
+				"type",
+				"value"
+			],
 			"properties": {
 				"format": {
 					"type": "string"
@@ -130,6 +135,11 @@
 		"biometricsType": {
 			"additionalProperties": false,
 			"type": "object",
+			"required": [
+				"format",
+				"version",
+				"value"
+			],
 			"properties": {
 				"format": {
 					"type": "string"
@@ -150,88 +160,471 @@
 			"type": "object",
 			"required": [
 				"IDSchemaVersion",
-				"fullName",
+				"name",
+				"surname",
 				"dateOfBirth",
 				"gender",
+				"placeOfBirth",
+				"divisionalSecretariatOfBirth",
 				"addressLine1",
-				"addressLine2",
-				"addressLine3",
-				"region",
 				"province",
-				"city",
-				"zone",
+				"district",
+				"divisionalSecretariat",
+				"grammaNiladhari",
 				"postalCode",
-				"phone",
-				"email",
-				"proofOfIdentity",
+				"applicantSignature",
 				"individualBiometrics"
 			],
 			"properties": {
-				"proofOfAddress": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"gender": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"city": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"postalCode": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^[(?i)A-Z0-9]{5}$|^NA$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
+				"IDSchemaVersion": {
+					"bioAttributes": [],
+					"fieldCategory": "none",
+					"format": "none",
+					"type": "number",
+					"fieldType": "default",
+					"minimum": 0
+				},
+				"UIN": {
+					"bioAttributes": [],
+					"fieldCategory": "none",
 					"format": "none",
 					"type": "string",
 					"fieldType": "default"
 				},
-				"proofOfException-1": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
+				"familyName": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{3,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"name": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{3,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"surname": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{3,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"gender": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"dateOfBirth": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"placeOfBirth": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{2,128}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"divisionalSecretariatOfBirth": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"deathDeclared": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(yes|no)$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"dateOfDeath": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"addressLine1": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,128}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"addressLine2": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"addressLine3": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"province": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"district": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"divisionalSecretariat": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"grammaNiladhari": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?=.{1,50}$).*",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"postalCode": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^[0-9]{5}$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"currentAddressLine1": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentAddressLine2": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentAddressLine3": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,128})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentProvince": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentDistrict": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentDivisionalSecretariat": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentGramaNiladhari": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(|.{1,50})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
+				},
+				"currentPostalCode": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^$|^[0-9]{5}$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
 				},
 				"referenceIdentityNumber": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^([0-9]{10,30})$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(?:\\d{9}[VXvx]|\\d{12})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "kyc",
 					"format": "kyc",
 					"type": "string",
 					"fieldType": "default"
+				},
+				"phone": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^(0?7[0-9]{8})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"email": {
+					"bioAttributes": [],
+					"validators": [
+						{
+							"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
+							"arguments": [],
+							"type": "regex"
+						}
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "default"
+				},
+				"preferredLang": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"type": "string",
+					"fieldType": "dynamic"
+				},
+				"applicantSignature": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"subType": "POI",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfDateOfBirth": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfAddress": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfIdentity": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfRelationship": {
+					"bioAttributes": [],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
+				},
+				"proofOfException": {
+					"bioAttributes": [],
+					"fieldCategory": "evidence",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/documentType"
 				},
 				"individualBiometrics": {
 					"bioAttributes": [
@@ -252,109 +645,49 @@
 					"fieldCategory": "pvt",
 					"format": "none",
 					"fieldType": "default",
-					"$ref": "#\/definitions\/biometricsType"
-				},
-				"province": {
+					"$ref": "#/definitions/biometricsType"
+				},
+				"individualAuthBiometrics": {
 					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"zone": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"proofOfDateOfBirth": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"addressLine1": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"addressLine2": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"residenceStatus": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "kyc",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"addressLine3": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"email": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
+						"leftEye",
+						"rightEye",
+						"rightIndex",
+						"rightLittle",
+						"rightRing",
+						"rightMiddle",
+						"leftIndex",
+						"leftLittle",
+						"leftRing",
+						"leftMiddle",
+						"leftThumb",
+						"rightThumb",
+						"face"
+					],
+					"fieldCategory": "pvt",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/biometricsType"
+				},
+				"introducerRID": {
+					"bioAttributes": [],
+					"fieldCategory": "evidence",
 					"format": "none",
 					"type": "string",
 					"fieldType": "default"
 				},
-				"introducerRID": {
-					"bioAttributes": [
-					],
+				"introducerUIN": {
+					"bioAttributes": [],
 					"fieldCategory": "evidence",
 					"format": "none",
 					"type": "string",
 					"fieldType": "default"
+				},
+				"introducerName": {
+					"bioAttributes": [],
+					"fieldCategory": "evidence",
+					"format": "none",
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
 				},
 				"introducerBiometrics": {
 					"bioAttributes": [
@@ -375,214 +708,8 @@
 					"fieldCategory": "pvt",
 					"format": "none",
 					"fieldType": "default",
-					"$ref": "#\/definitions\/biometricsType"
-				},
-				"fullName": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"dateOfBirth": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])\/([0][1-9]|1[0-2])\/([0][1-9]|[1-2][0-9]|3[01])$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"individualAuthBiometrics": {
-					"bioAttributes": [
-						"leftEye",
-						"rightEye",
-						"rightIndex",
-						"rightLittle",
-						"rightRing",
-						"rightMiddle",
-						"leftIndex",
-						"leftLittle",
-						"leftRing",
-						"leftMiddle",
-						"leftThumb",
-						"rightThumb",
-						"face"
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/biometricsType"
-				},
-				"introducerUIN": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"proofOfIdentity": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"IDSchemaVersion": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "none",
-					"format": "none",
-					"type": "number",
-					"fieldType": "default",
-					"minimum": 0
-				},
-				"proofOfException": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"phone": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^[+]*([0-9]{1})([0-9]{9})$",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"introducerName": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "evidence",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"proofOfRelationship": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/documentType"
-				},
-				"UIN": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "none",
-					"format": "none",
-					"type": "string",
-					"fieldType": "default"
-				},
-				"preferredLang": {
-					"bioAttributes": [
-					],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"type": "string",
-					"fieldType": "dynamic"
-				},
-				"region": {
-					"bioAttributes": [
-					],
-					"validators": [{
-						"validator": "^(?=.{0,50}$).*",
-						"arguments": [
-						],
-						"type": "regex"
-					}],
-					"fieldCategory": "pvt",
-					"format": "none",
-					"fieldType": "default",
-					"$ref": "#\/definitions\/simpleType"
-				},
-				"introducerInfoToken": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "evidence",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "deceasedInformer": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "evidence",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "deceasedDeclarationDate": {
-                    "bioAttributes": [
-                    ],
-                    "validators": [
-                        {
-                            "validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
-                            "arguments": [
-                            ],
-                            "type": "regex"
-                        }
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "declaredAsDeceased": {
-                    "bioAttributes": [
-                    ],
-                    "validators": [
-                        {
-                            "validator": "^(Y|N)$",
-                            "arguments": [
-                            ],
-                            "type": "regex"
-                        }
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-                "typeOfDeath": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                },
-				"packetCreatedOn": {
-                    "bioAttributes": [
-                    ],
-                    "fieldCategory": "pvt",
-                    "format": "none",
-                    "type": "string",
-                    "fieldType": "default"
-                }
+					"$ref": "#/definitions/biometricsType"
+				}
 			}
 		}
 	}
@@ -678,9 +805,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -718,7 +845,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -824,7 +951,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -966,7 +1093,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -975,23 +1102,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AMJ3"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.453125" style="1"/>
-    <col min="2" max="2" width="8.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="11.54296875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.453125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.44140625" style="1"/>
+    <col min="2" max="2" width="8.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="31" style="1" customWidth="1"/>
-    <col min="6" max="6" width="53.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7265625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="53.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.44140625" style="2" customWidth="1"/>
     <col min="9" max="9" width="10" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" style="2"/>
-    <col min="11" max="1023" width="8.453125" style="1"/>
-    <col min="1024" max="1024" width="11.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.44140625" style="2"/>
+    <col min="11" max="1023" width="8.44140625" style="1"/>
+    <col min="1024" max="1024" width="11.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1023,7 +1150,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1055,7 +1182,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="F3" s="5"/>
     </row>

</xml_diff>